<commit_message>
Catch the methods that blow up upwards, not just downwards
The negative-SPPR flag missed the Bay of Bengal, where `sym_GE_asDC`
returns 2.1e13 tonnes and `sym_TE_asDC` 1.5e13 - positive, so nothing
objected, and 6,700 times the trophic-chain estimate. After the usual 9:1
wet-weight-to-carbon conversion that is some thousands of times the entire
annual primary production of that sea, which is a near-singular solve
rather than a modelling difference.

Across the healthy models the network methods run 0.1x to 4.6x the
trophic-chain estimate, so the threshold sits at 25x. It flags the two Bay
of Bengal solves and `MC_new_TE_EEfix` on the Okhotsk model at 76x, and
leaves everything else alone. The flagged rows stay in the sheet - this is
a plausibility flag, not a verdict on which method is right - but the
Summary sheet will no longer lead with one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/LME_052/models/52_1_Sea_of_Okhotsk_NE_(1980).xlsx
+++ b/data/LME_052/models/52_1_Sea_of_Okhotsk_NE_(1980).xlsx
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -58175,14 +58175,14 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>MC_new_TE_EEfix</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>ok</t>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>IMPLAUSIBLE - up to 76x the trophic-chain estimate; the solve is near-singular for this model</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -58406,7 +58406,7 @@
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>6 of 20 methods are flagged above. A flagged row is a property of this model under that method, not of the mapping; see model_health in the SPPR workbook.</t>
+          <t>7 of 20 methods are flagged above. A flagged row is a property of this model under that method, not of the mapping; see model_health in the SPPR workbook.</t>
         </is>
       </c>
     </row>

</xml_diff>